<commit_message>
Update Philly BYOB Restaurant google form.xlsx
</commit_message>
<xml_diff>
--- a/philly_yelp_crawler/data/Philly BYOB Restaurant google form.xlsx
+++ b/philly_yelp_crawler/data/Philly BYOB Restaurant google form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slow3\OneDrive\桌面\GitHubProjects\BYOB\philly_yelp_crawler\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59AFE7EE-A7E9-4F06-95A7-A95CA5F9D75F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D8F82C-812A-4E42-8337-E0E030EF44A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{888A9BF0-2D43-4E31-B177-D5314CD5866A}"/>
   </bookViews>
@@ -161,9 +161,6 @@
     <t>6118 Ridge Ave, Philadelphia, PA 19128</t>
   </si>
   <si>
-    <t>1247 S 13th St</t>
-  </si>
-  <si>
     <t xml:space="preserve">(215) 606-1899  </t>
   </si>
   <si>
@@ -213,6 +210,9 @@
   </si>
   <si>
     <t xml:space="preserve">(215) 465-2200  </t>
+  </si>
+  <si>
+    <t>1247 S 13th St, Philadelphia, PA 19147</t>
   </si>
 </sst>
 </file>
@@ -635,7 +635,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -654,7 +654,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -665,7 +665,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -676,7 +676,7 @@
         <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -687,7 +687,7 @@
         <v>17</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -698,7 +698,7 @@
         <v>19</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -709,7 +709,7 @@
         <v>21</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -720,7 +720,7 @@
         <v>23</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -731,7 +731,7 @@
         <v>25</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -742,7 +742,7 @@
         <v>19</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -753,7 +753,7 @@
         <v>27</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -764,7 +764,7 @@
         <v>29</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -775,7 +775,7 @@
         <v>31</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -786,7 +786,7 @@
         <v>33</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -797,7 +797,7 @@
         <v>35</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -808,7 +808,7 @@
         <v>37</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -819,7 +819,7 @@
         <v>5</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -830,7 +830,7 @@
         <v>39</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -838,10 +838,10 @@
         <v>3</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>